<commit_message>
Update unit mismatch files with new data and format changes
- Updated the unit-mismatches CSV file to include a new column for file names, enhancing data tracking.
- Modified the unit-mismatches Excel files to reflect the latest changes in the CSV data.
</commit_message>
<xml_diff>
--- a/data/transactions/_unit-mismatches/unit-mismatches.xlsx
+++ b/data/transactions/_unit-mismatches/unit-mismatches.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>الكود</t>
   </si>
@@ -29,13 +29,70 @@
   </si>
   <si>
     <t>آخر رقم فاتورة</t>
+  </si>
+  <si>
+    <t>اسم الملف</t>
+  </si>
+  <si>
+    <t>10106040</t>
+  </si>
+  <si>
+    <t>فريون 1ك R134</t>
+  </si>
+  <si>
+    <t>عدد</t>
+  </si>
+  <si>
+    <t>كيلو</t>
+  </si>
+  <si>
+    <t>الفاروق</t>
+  </si>
+  <si>
+    <t>2437</t>
+  </si>
+  <si>
+    <t>أذونات الإضافة لشهر 3.xlsx</t>
+  </si>
+  <si>
+    <t>10801007</t>
+  </si>
+  <si>
+    <t>خشب شوايه فلندي 3/4 ×4</t>
+  </si>
+  <si>
+    <t>متر³</t>
+  </si>
+  <si>
+    <t>متر 2</t>
+  </si>
+  <si>
+    <t>اخشاب النعام</t>
+  </si>
+  <si>
+    <t>783</t>
+  </si>
+  <si>
+    <t>11404002</t>
+  </si>
+  <si>
+    <t>خوصة حديد 20 × 40 مم × 6 م</t>
+  </si>
+  <si>
+    <t>الاسراء</t>
+  </si>
+  <si>
+    <t>709</t>
+  </si>
+  <si>
+    <t>أذونات الإضافة لشهر 6.xlsx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -49,8 +106,12 @@
       <sz val="12"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -60,6 +121,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,10 +156,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -437,7 +515,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -446,9 +524,10 @@
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -467,9 +546,81 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:G4"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Update unit mismatch files with new data and remove obsolete entry
- Updated the unit-mismatches CSV file by removing an obsolete entry for a specific item.
- Modified the unit-mismatches Excel files to reflect the latest changes in the CSV data.
</commit_message>
<xml_diff>
--- a/data/transactions/_unit-mismatches/unit-mismatches.xlsx
+++ b/data/transactions/_unit-mismatches/unit-mismatches.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>الكود</t>
   </si>
@@ -71,21 +71,6 @@
   </si>
   <si>
     <t>783</t>
-  </si>
-  <si>
-    <t>11404002</t>
-  </si>
-  <si>
-    <t>خوصة حديد 20 × 40 مم × 6 م</t>
-  </si>
-  <si>
-    <t>الاسراء</t>
-  </si>
-  <si>
-    <t>709</t>
-  </si>
-  <si>
-    <t>أذونات الإضافة لشهر 6.xlsx</t>
   </si>
 </sst>
 </file>
@@ -515,7 +500,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -596,31 +581,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G3"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Update unit mismatches files with revised data in Excel and CSV formats
</commit_message>
<xml_diff>
--- a/data/transactions/_unit-mismatches/unit-mismatches.xlsx
+++ b/data/transactions/_unit-mismatches/unit-mismatches.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>الكود</t>
   </si>
@@ -32,52 +32,13 @@
   </si>
   <si>
     <t>اسم الملف</t>
-  </si>
-  <si>
-    <t>10106040</t>
-  </si>
-  <si>
-    <t>فريون 1ك R134</t>
-  </si>
-  <si>
-    <t>عدد</t>
-  </si>
-  <si>
-    <t>كيلو</t>
-  </si>
-  <si>
-    <t>الفاروق</t>
-  </si>
-  <si>
-    <t>2437</t>
-  </si>
-  <si>
-    <t>أذونات الإضافة لشهر 3.xlsx</t>
-  </si>
-  <si>
-    <t>10801007</t>
-  </si>
-  <si>
-    <t>خشب شوايه فلندي 3/4 ×4</t>
-  </si>
-  <si>
-    <t>متر³</t>
-  </si>
-  <si>
-    <t>متر 2</t>
-  </si>
-  <si>
-    <t>اخشاب النعام</t>
-  </si>
-  <si>
-    <t>783</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -91,12 +52,8 @@
       <sz val="12"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -106,11 +63,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1E3A5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -141,22 +93,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -500,7 +440,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="22" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -535,54 +475,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G1"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>